<commit_message>
data: synchronize D365 PQU schedule from Microsoft
</commit_message>
<xml_diff>
--- a/excel/D365-PQU-Tracker.xlsx
+++ b/excel/D365-PQU-Tracker.xlsx
@@ -865,7 +865,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
@@ -1192,14 +1192,14 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -1220,14 +1220,14 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -1248,14 +1248,14 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1276,14 +1276,14 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -1304,14 +1304,14 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1332,14 +1332,14 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -1360,14 +1360,14 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1388,14 +1388,14 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -1416,14 +1416,14 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1444,14 +1444,14 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -1472,14 +1472,14 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -1500,14 +1500,14 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -1528,14 +1528,14 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -1556,14 +1556,14 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -1584,14 +1584,14 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -1612,14 +1612,14 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -1640,14 +1640,14 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -1668,14 +1668,14 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -1696,14 +1696,14 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -1724,14 +1724,14 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1752,14 +1752,14 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -1780,14 +1780,14 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1808,14 +1808,14 @@
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1836,14 +1836,14 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1864,14 +1864,14 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1892,14 +1892,14 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1920,14 +1920,14 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1948,14 +1948,14 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1976,14 +1976,14 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -2004,14 +2004,14 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2032,14 +2032,14 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2060,14 +2060,14 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2088,14 +2088,14 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2116,14 +2116,14 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2144,14 +2144,14 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2172,14 +2172,14 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2200,14 +2200,14 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2228,14 +2228,14 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2256,14 +2256,14 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2284,14 +2284,14 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2312,14 +2312,14 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2340,14 +2340,14 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2368,14 +2368,14 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2396,14 +2396,14 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2424,14 +2424,14 @@
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2452,14 +2452,14 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2480,14 +2480,14 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2508,14 +2508,14 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2536,14 +2536,14 @@
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2564,14 +2564,14 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2592,14 +2592,14 @@
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2620,14 +2620,14 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2648,14 +2648,14 @@
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2676,14 +2676,14 @@
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2704,14 +2704,14 @@
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -2732,14 +2732,14 @@
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -2760,14 +2760,14 @@
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -2788,14 +2788,14 @@
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/MicrosoftDocs/dynamics-365-unified-operations-public/deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd/articles/fin-ops-core/dev-itpro/get-started/quality-updates-schedule.md</t>
+          <t>https://raw.githubusercontent.com/MicrosoftDocs/dynamics-365-unified-operations-public/b9cc4ebd5957b88060059dc2a7e3b08364ab3dca/articles/fin-ops-core/dev-itpro/get-started/quality-updates-schedule.md</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948+00:00</t>
+          <t>2026-09-25T05:02:58.124992+00:00</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
     </row>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:45.947948Z</t>
+          <t>2026-09-25T05:02:58.124992Z</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -3557,7 +3557,7 @@
       </c>
       <c r="O2" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P2" s="7" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P3" s="7" t="inlineStr">
@@ -3713,7 +3713,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P4" s="7" t="inlineStr">
@@ -3791,7 +3791,7 @@
       </c>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P6" s="7" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P8" s="7" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P10" s="7" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="O11" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P11" s="7" t="inlineStr">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P12" s="7" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="O13" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P13" s="7" t="inlineStr">
@@ -4489,7 +4489,7 @@
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P14" s="7" t="inlineStr">
@@ -4567,7 +4567,7 @@
       </c>
       <c r="O15" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P15" s="7" t="inlineStr">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="O16" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P16" s="7" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="O17" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P17" s="7" t="inlineStr">
@@ -4801,7 +4801,7 @@
       </c>
       <c r="O18" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P18" s="7" t="inlineStr">
@@ -4879,7 +4879,7 @@
       </c>
       <c r="O19" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P19" s="7" t="inlineStr">
@@ -4957,7 +4957,7 @@
       </c>
       <c r="O20" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P20" s="7" t="inlineStr">
@@ -5039,7 +5039,7 @@
       </c>
       <c r="O21" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P21" s="7" t="inlineStr">
@@ -5121,7 +5121,7 @@
       </c>
       <c r="O22" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P22" s="7" t="inlineStr">
@@ -5191,7 +5191,7 @@
       </c>
       <c r="O23" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P23" s="7" t="inlineStr">
@@ -5261,7 +5261,7 @@
       </c>
       <c r="O24" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P24" s="7" t="inlineStr">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="O25" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P25" s="7" t="inlineStr">
@@ -5401,7 +5401,7 @@
       </c>
       <c r="O26" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P26" s="7" t="inlineStr">
@@ -5479,7 +5479,7 @@
       </c>
       <c r="O27" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P27" s="7" t="inlineStr">
@@ -5557,7 +5557,7 @@
       </c>
       <c r="O28" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P28" s="7" t="inlineStr">
@@ -5635,7 +5635,7 @@
       </c>
       <c r="O29" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P29" s="7" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="O30" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P30" s="7" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="O31" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P31" s="7" t="inlineStr">
@@ -5877,7 +5877,7 @@
       </c>
       <c r="O32" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P32" s="7" t="inlineStr">
@@ -5947,7 +5947,7 @@
       </c>
       <c r="O33" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P33" s="7" t="inlineStr">
@@ -6017,7 +6017,7 @@
       </c>
       <c r="O34" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P34" s="7" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="O35" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P35" s="7" t="inlineStr">
@@ -6157,7 +6157,7 @@
       </c>
       <c r="O36" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P36" s="7" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="O37" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P37" s="7" t="inlineStr">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="O38" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P38" s="7" t="inlineStr">
@@ -6367,7 +6367,7 @@
       </c>
       <c r="O39" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P39" s="7" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="O40" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P40" s="7" t="inlineStr">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="O41" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P41" s="7" t="inlineStr">
@@ -6577,7 +6577,7 @@
       </c>
       <c r="O42" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P42" s="7" t="inlineStr">
@@ -6647,7 +6647,7 @@
       </c>
       <c r="O43" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P43" s="7" t="inlineStr">
@@ -6717,7 +6717,7 @@
       </c>
       <c r="O44" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P44" s="7" t="inlineStr">
@@ -6787,7 +6787,7 @@
       </c>
       <c r="O45" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P45" s="7" t="inlineStr">
@@ -6857,7 +6857,7 @@
       </c>
       <c r="O46" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P46" s="7" t="inlineStr">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="O47" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P47" s="7" t="inlineStr">
@@ -6997,7 +6997,7 @@
       </c>
       <c r="O48" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P48" s="7" t="inlineStr">
@@ -7067,7 +7067,7 @@
       </c>
       <c r="O49" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P49" s="7" t="inlineStr">
@@ -7137,7 +7137,7 @@
       </c>
       <c r="O50" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P50" s="7" t="inlineStr">
@@ -7207,7 +7207,7 @@
       </c>
       <c r="O51" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P51" s="7" t="inlineStr">
@@ -7277,7 +7277,7 @@
       </c>
       <c r="O52" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P52" s="7" t="inlineStr">
@@ -7347,7 +7347,7 @@
       </c>
       <c r="O53" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P53" s="7" t="inlineStr">
@@ -7417,7 +7417,7 @@
       </c>
       <c r="O54" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P54" s="7" t="inlineStr">
@@ -7487,7 +7487,7 @@
       </c>
       <c r="O55" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P55" s="7" t="inlineStr">
@@ -7557,7 +7557,7 @@
       </c>
       <c r="O56" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P56" s="7" t="inlineStr">
@@ -7627,7 +7627,7 @@
       </c>
       <c r="O57" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P57" s="7" t="inlineStr">
@@ -7697,7 +7697,7 @@
       </c>
       <c r="O58" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P58" s="7" t="inlineStr">
@@ -7767,7 +7767,7 @@
       </c>
       <c r="O59" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P59" s="7" t="inlineStr">
@@ -7837,7 +7837,7 @@
       </c>
       <c r="O60" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P60" s="7" t="inlineStr">
@@ -8050,7 +8050,7 @@
       </c>
       <c r="O2" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P2" s="7" t="inlineStr">
@@ -8132,7 +8132,7 @@
       </c>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P3" s="7" t="inlineStr">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P4" s="7" t="inlineStr">
@@ -8296,7 +8296,7 @@
       </c>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
@@ -8378,7 +8378,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P6" s="7" t="inlineStr">
@@ -8579,7 +8579,7 @@
       </c>
       <c r="O2" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P2" s="7" t="inlineStr">
@@ -8649,7 +8649,7 @@
       </c>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P3" s="7" t="inlineStr">
@@ -8719,7 +8719,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P4" s="7" t="inlineStr">
@@ -8789,7 +8789,7 @@
       </c>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
@@ -8859,7 +8859,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P6" s="7" t="inlineStr">
@@ -8929,7 +8929,7 @@
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
@@ -8999,7 +8999,7 @@
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P8" s="7" t="inlineStr">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
@@ -9139,7 +9139,7 @@
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P10" s="7" t="inlineStr">
@@ -9209,7 +9209,7 @@
       </c>
       <c r="O11" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P11" s="7" t="inlineStr">
@@ -9279,7 +9279,7 @@
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P12" s="7" t="inlineStr">
@@ -9349,7 +9349,7 @@
       </c>
       <c r="O13" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P13" s="7" t="inlineStr">
@@ -9419,7 +9419,7 @@
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P14" s="7" t="inlineStr">
@@ -9489,7 +9489,7 @@
       </c>
       <c r="O15" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P15" s="7" t="inlineStr">
@@ -9559,7 +9559,7 @@
       </c>
       <c r="O16" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P16" s="7" t="inlineStr">
@@ -9629,7 +9629,7 @@
       </c>
       <c r="O17" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P17" s="7" t="inlineStr">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="O18" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P18" s="7" t="inlineStr">
@@ -9769,7 +9769,7 @@
       </c>
       <c r="O19" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P19" s="7" t="inlineStr">
@@ -9839,7 +9839,7 @@
       </c>
       <c r="O20" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P20" s="7" t="inlineStr">
@@ -9909,7 +9909,7 @@
       </c>
       <c r="O21" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P21" s="7" t="inlineStr">
@@ -9979,7 +9979,7 @@
       </c>
       <c r="O22" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P22" s="7" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="O23" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P23" s="7" t="inlineStr">
@@ -10119,7 +10119,7 @@
       </c>
       <c r="O24" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P24" s="7" t="inlineStr">
@@ -10189,7 +10189,7 @@
       </c>
       <c r="O25" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P25" s="7" t="inlineStr">
@@ -10259,7 +10259,7 @@
       </c>
       <c r="O26" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P26" s="7" t="inlineStr">
@@ -10329,7 +10329,7 @@
       </c>
       <c r="O27" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P27" s="7" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="O28" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P28" s="7" t="inlineStr">
@@ -10469,7 +10469,7 @@
       </c>
       <c r="O29" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P29" s="7" t="inlineStr">
@@ -10539,7 +10539,7 @@
       </c>
       <c r="O30" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P30" s="7" t="inlineStr">
@@ -10609,7 +10609,7 @@
       </c>
       <c r="O31" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P31" s="7" t="inlineStr">
@@ -10679,7 +10679,7 @@
       </c>
       <c r="O32" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P32" s="7" t="inlineStr">
@@ -10749,7 +10749,7 @@
       </c>
       <c r="O33" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
       <c r="P33" s="7" t="inlineStr">
@@ -10885,7 +10885,7 @@
       <c r="I2" s="7" t="n"/>
       <c r="J2" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -10927,7 +10927,7 @@
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -10969,7 +10969,7 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11011,7 +11011,7 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11053,7 +11053,7 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11095,7 +11095,7 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11133,7 +11133,7 @@
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11175,7 +11175,7 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11217,7 +11217,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11259,7 +11259,7 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11301,7 +11301,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11343,7 +11343,7 @@
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11381,7 +11381,7 @@
       <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11423,7 +11423,7 @@
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11465,7 +11465,7 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11507,7 +11507,7 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11549,7 +11549,7 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11591,7 +11591,7 @@
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11629,7 +11629,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11671,7 +11671,7 @@
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11713,7 +11713,7 @@
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11755,7 +11755,7 @@
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11797,7 +11797,7 @@
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11839,7 +11839,7 @@
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11877,7 +11877,7 @@
       <c r="I26" s="7" t="n"/>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11919,7 +11919,7 @@
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -11961,7 +11961,7 @@
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -12003,7 +12003,7 @@
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -12045,7 +12045,7 @@
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>
@@ -12087,7 +12087,7 @@
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>deb37ecf6bc37a4862d78515fa35d8a4dc38bcdd</t>
+          <t>b9cc4ebd5957b88060059dc2a7e3b08364ab3dca</t>
         </is>
       </c>
     </row>

</xml_diff>